<commit_message>
feat: wire master mechanics and roster quality
</commit_message>
<xml_diff>
--- a/xlsx/ysbzs_v1_linked_data_tables.xlsx
+++ b/xlsx/ysbzs_v1_linked_data_tables.xlsx
@@ -36,7 +36,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_遗物祝福_好读版'!$A$1:$P$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_形状行动槽_好读版'!$A$1:$T$128</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_跨表校验'!$A$1:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'10_初始阵容'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'10_初始阵容'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'11_英雄领域_联动版'!$A$1:$I$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'12_元素反应_联动版'!$A$1:$H$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'13_第7天兽群试炼_联动版'!$A$1:$Q$10</definedName>
@@ -1807,7 +1807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1816,7 +1816,8 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1837,20 +1838,25 @@
       </c>
       <c r="D1" s="32" t="inlineStr">
         <is>
+          <t>品质覆盖</t>
+        </is>
+      </c>
+      <c r="E1" s="32" t="inlineStr">
+        <is>
           <t>行(1-8)</t>
         </is>
       </c>
-      <c r="E1" s="32" t="inlineStr">
+      <c r="F1" s="32" t="inlineStr">
         <is>
           <t>列(1-8)</t>
         </is>
       </c>
-      <c r="F1" s="32" t="inlineStr">
+      <c r="G1" s="32" t="inlineStr">
         <is>
           <t>启用</t>
         </is>
       </c>
-      <c r="G1" s="32" t="inlineStr">
+      <c r="H1" s="32" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1874,22 +1880,27 @@
       </c>
       <c r="D2" s="33" t="inlineStr">
         <is>
+          <t>黄金</t>
+        </is>
+      </c>
+      <c r="E2" s="33" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E2" s="33" t="inlineStr">
+      <c r="F2" s="33" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F2" s="33" t="inlineStr">
+      <c r="G2" s="33" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="G2" s="33" t="inlineStr">
-        <is>
-          <t>第7天火核心：融焰娘，品质覆盖=黄金，实际快照见13</t>
+      <c r="H2" s="33" t="inlineStr">
+        <is>
+          <t>第7天火核心：融焰娘，实际快照见13</t>
         </is>
       </c>
     </row>
@@ -1911,22 +1922,27 @@
       </c>
       <c r="D3" s="33" t="inlineStr">
         <is>
+          <t>白银</t>
+        </is>
+      </c>
+      <c r="E3" s="33" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E3" s="33" t="inlineStr">
+      <c r="F3" s="33" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F3" s="33" t="inlineStr">
+      <c r="G3" s="33" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="G3" s="33" t="inlineStr">
-        <is>
-          <t>火绒狐，品质覆盖=白银，实际快照见13</t>
+      <c r="H3" s="33" t="inlineStr">
+        <is>
+          <t>火绒狐，实际快照见13</t>
         </is>
       </c>
     </row>
@@ -1948,22 +1964,27 @@
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
+          <t>白银</t>
+        </is>
+      </c>
+      <c r="E4" s="33" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E4" s="33" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F4" s="33" t="inlineStr">
+      <c r="G4" s="33" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="G4" s="33" t="inlineStr">
-        <is>
-          <t>冲浪鸭，品质覆盖=白银，实际快照见13</t>
+      <c r="H4" s="33" t="inlineStr">
+        <is>
+          <t>冲浪鸭，实际快照见13</t>
         </is>
       </c>
     </row>
@@ -1985,27 +2006,32 @@
       </c>
       <c r="D5" s="33" t="inlineStr">
         <is>
+          <t>白银</t>
+        </is>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E5" s="33" t="inlineStr">
+      <c r="F5" s="33" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F5" s="33" t="inlineStr">
+      <c r="G5" s="33" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="G5" s="33" t="inlineStr">
-        <is>
-          <t>疾风隼，承接旋风狸风聚火功能，品质覆盖=白银，实际快照见13</t>
+      <c r="H5" s="33" t="inlineStr">
+        <is>
+          <t>疾风隼，承接旋风狸风聚火功能，实际快照见13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:H5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>